<commit_message>
Update coding question templates and documentation
</commit_message>
<xml_diff>
--- a/public/templates/coding_questions_template.xlsx
+++ b/public/templates/coding_questions_template.xlsx
@@ -397,221 +397,147 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:R2"/>
+  <cols>
+    <col min="1" max="1" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Question Type</v>
+        <v>Problem Statement</v>
       </c>
       <c r="B1" t="str">
-        <v>Question Text</v>
+        <v>Section Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Explanation</v>
+        <v>Difficulty</v>
       </c>
       <c r="D1" t="str">
         <v>Score Points</v>
       </c>
       <c r="E1" t="str">
-        <v>Test Cases JSON</v>
+        <v>Time Limit</v>
       </c>
       <c r="F1" t="str">
-        <v>Difficulty</v>
+        <v>Constraints</v>
       </c>
       <c r="G1" t="str">
-        <v>Concept</v>
+        <v>Sample Input 1</v>
       </c>
       <c r="H1" t="str">
-        <v>Company Name</v>
+        <v>Sample Output 1</v>
       </c>
       <c r="I1" t="str">
-        <v>Exam Name</v>
+        <v>Sample Input 2</v>
       </c>
       <c r="J1" t="str">
-        <v>Exam Year</v>
+        <v>Sample Output 2</v>
       </c>
       <c r="K1" t="str">
-        <v>Section Name</v>
+        <v>Sample Input 3</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Sample Output 3</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Hidden Input 1</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Hidden Output 1</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Hidden Input 2</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Hidden Output 2</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Hidden Input 3</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Hidden Output 3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>Coding Question</v>
+        <v>Write a program to reverse an array.</v>
       </c>
       <c r="B2" t="str">
-        <v>Write a function to add two numbers</v>
+        <v>Coding</v>
       </c>
       <c r="C2" t="str">
-        <v>The function should take two parameters and return their sum. Example: add(2, 3) should return 5</v>
+        <v>Medium</v>
       </c>
       <c r="D2">
-        <v>10</v>
-      </c>
-      <c r="E2" t="str">
-        <v>[{"input":"2, 3","expectedOutput":"5","explanation":"2 + 3 = 5"},{"input":"10, 20","expectedOutput":"30","explanation":"10 + 20 = 30"},{"input":"-5, 5","expectedOutput":"0","explanation":"-5 + 5 = 0"}]</v>
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
       </c>
       <c r="F2" t="str">
-        <v>easy</v>
-      </c>
-      <c r="G2" t="str">
-        <v>programming</v>
+        <v>1 &lt;= N &lt;= 10^5</v>
+      </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">5
+1 2 3 4 5</v>
       </c>
       <c r="H2" t="str">
-        <v>tcs</v>
-      </c>
-      <c r="I2" t="str">
-        <v>nqt</v>
+        <v>5 4 3 2 1</v>
+      </c>
+      <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">3
+1 2 3</v>
       </c>
       <c r="J2" t="str">
-        <v>2025</v>
+        <v>3 2 1</v>
       </c>
       <c r="K2" t="str">
-        <v>coding</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Coding Question</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Write a function to check if a number is even</v>
-      </c>
-      <c r="C3" t="str">
-        <v>The function should return true if the number is even, false otherwise. A number is even if it's divisible by 2</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3" t="str">
-        <v>[{"input":"4","expectedOutput":"true","explanation":"4 is divisible by 2"},{"input":"7","expectedOutput":"false","explanation":"7 is not divisible by 2"},{"input":"0","expectedOutput":"true","explanation":"0 is considered even"}]</v>
-      </c>
-      <c r="F3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="G3" t="str">
-        <v>logical</v>
-      </c>
-      <c r="H3" t="str">
-        <v>infosys, wipro</v>
-      </c>
-      <c r="I3" t="str">
-        <v>infytq, wiprotest</v>
-      </c>
-      <c r="J3" t="str">
-        <v>2025, 2026</v>
-      </c>
-      <c r="K3" t="str">
-        <v>coding, technical</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Coding Question</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Write a function to find the maximum of two numbers</v>
-      </c>
-      <c r="C4" t="str">
-        <v>The function should compare two numbers and return the larger one. If equal, return either</v>
-      </c>
-      <c r="D4">
-        <v>8</v>
-      </c>
-      <c r="E4" t="str">
-        <v>[{"input":"5, 10","expectedOutput":"10","explanation":"10 is greater than 5"},{"input":"15, 8","expectedOutput":"15","explanation":"15 is greater than 8"},{"input":"7, 7","expectedOutput":"7","explanation":"Both numbers are equal"}]</v>
-      </c>
-      <c r="F4" t="str">
-        <v>hard</v>
-      </c>
-      <c r="G4" t="str">
-        <v>math</v>
-      </c>
-      <c r="H4" t="str">
-        <v>cognizant</v>
-      </c>
-      <c r="I4" t="str">
-        <v>genC</v>
-      </c>
-      <c r="J4" t="str">
-        <v>2026</v>
-      </c>
-      <c r="K4" t="str">
-        <v>logical</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Coding Question</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Write a function to reverse a string</v>
-      </c>
-      <c r="C5" t="str">
-        <v>The function should take a string as input and return the reversed string. Example: reverse('hello') should return 'olleh'</v>
-      </c>
-      <c r="D5">
-        <v>12</v>
-      </c>
-      <c r="E5" t="str">
-        <v>[{"input":"hello","expectedOutput":"olleh","explanation":"Reverse of hello is olleh"},{"input":"world","expectedOutput":"dlrow","explanation":"Reverse of world is dlrow"},{"input":"a","expectedOutput":"a","explanation":"Single character remains same"}]</v>
-      </c>
-      <c r="F5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="G5" t="str">
-        <v>fundamentals</v>
-      </c>
-      <c r="H5" t="str">
-        <v>amazon</v>
-      </c>
-      <c r="I5" t="str">
-        <v>aws-cert</v>
-      </c>
-      <c r="J5" t="str">
-        <v>2024</v>
-      </c>
-      <c r="K5" t="str">
-        <v>verbal</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Coding Question</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Write a function to calculate factorial</v>
-      </c>
-      <c r="C6" t="str">
-        <v>The function should calculate the factorial of a non-negative integer. Factorial of n is n! = n × (n-1) × (n-2) × ... × 1</v>
-      </c>
-      <c r="D6">
-        <v>15</v>
-      </c>
-      <c r="E6" t="str">
-        <v>[{"input":"5","expectedOutput":"120","explanation":"5! = 5 × 4 × 3 × 2 × 1 = 120"},{"input":"3","expectedOutput":"6","explanation":"3! = 3 × 2 × 1 = 6"},{"input":"0","expectedOutput":"1","explanation":"0! is defined as 1"}]</v>
-      </c>
-      <c r="F6" t="str">
-        <v>easy</v>
-      </c>
-      <c r="G6" t="str">
-        <v>science</v>
-      </c>
-      <c r="H6" t="str">
-        <v>google, microsoft</v>
-      </c>
-      <c r="I6" t="str">
-        <v>g-kickstart, ms-codility</v>
-      </c>
-      <c r="J6" t="str">
-        <v>2024, 2025</v>
-      </c>
-      <c r="K6" t="str">
-        <v>algorithms, technical</v>
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str" xml:space="preserve">
+        <v xml:space="preserve">4
+9 8 7 6</v>
+      </c>
+      <c r="N2" t="str">
+        <v>6 7 8 9</v>
+      </c>
+      <c r="O2" t="str" xml:space="preserve">
+        <v xml:space="preserve">2
+1 1</v>
+      </c>
+      <c r="P2" t="str">
+        <v>1 1</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>